<commit_message>
Regenerate the Tupelo packet against the trimmed capture sheet
Same 33 screens, 27 venues, 27 stops, 27 labels and 22 over-target readings
as the 2026-08-04 build. The brief now runs five steps instead of six and
leads with the introduction, the field sheet carries 16 columns instead of
18, and the labels say PROPERTY OF MCTV DIGITAL with a phone number.
</commit_message>
<xml_diff>
--- a/docs/audits/tupelo-2026-08/MCTV_FieldSheet_Tupelo.xlsx
+++ b/docs/audits/tupelo-2026-08/MCTV_FieldSheet_Tupelo.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Field Sheet'!$A$1:$AC$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Field Sheet'!$A$1:$AA$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC34"/>
+  <dimension ref="A1:AA34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -496,24 +496,22 @@
     <col width="38" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="10" customWidth="1" min="16" max="16"/>
-    <col width="13" customWidth="1" min="17" max="17"/>
-    <col width="16" customWidth="1" min="18" max="18"/>
-    <col width="16" customWidth="1" min="19" max="19"/>
-    <col width="20" customWidth="1" min="20" max="20"/>
-    <col width="18" customWidth="1" min="21" max="21"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="15" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="34" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
     <col width="16" customWidth="1" min="22" max="22"/>
-    <col width="14" customWidth="1" min="23" max="23"/>
-    <col width="14" customWidth="1" min="24" max="24"/>
-    <col width="34" customWidth="1" min="25" max="25"/>
-    <col width="13" customWidth="1" min="26" max="26"/>
-    <col width="16" customWidth="1" min="27" max="27"/>
-    <col width="12" customWidth="1" min="28" max="28"/>
-    <col width="40" customWidth="1" min="29" max="29"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="10" customWidth="1" min="24" max="24"/>
+    <col width="40" customWidth="1" min="25" max="25"/>
+    <col width="16" customWidth="1" min="26" max="26"/>
+    <col width="12" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -574,92 +572,82 @@
       </c>
       <c r="L1" s="2" t="inlineStr">
         <is>
+          <t>Spoke with</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Card left?</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
           <t>Screen on?</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>Content playing?</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="P1" s="2" t="inlineStr">
+        <is>
+          <t>Power test OK?</t>
+        </is>
+      </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>Connection</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>Presentation OK?</t>
+        </is>
+      </c>
+      <c r="S1" s="2" t="inlineStr">
+        <is>
+          <t>Photos taken?</t>
+        </is>
+      </c>
+      <c r="T1" s="2" t="inlineStr">
+        <is>
+          <t>License # confirmed</t>
+        </is>
+      </c>
+      <c r="U1" s="2" t="inlineStr">
+        <is>
+          <t>Label applied?</t>
+        </is>
+      </c>
+      <c r="V1" s="2" t="inlineStr">
         <is>
           <t>Display brand</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="W1" s="2" t="inlineStr">
         <is>
           <t>Display model</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="X1" s="2" t="inlineStr">
         <is>
           <t>Size (in)</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
-        <is>
-          <t>Orientation</t>
-        </is>
-      </c>
-      <c r="R1" s="2" t="inlineStr">
-        <is>
-          <t>Mount type</t>
-        </is>
-      </c>
-      <c r="S1" s="2" t="inlineStr">
-        <is>
-          <t>Pi model</t>
-        </is>
-      </c>
-      <c r="T1" s="2" t="inlineStr">
-        <is>
-          <t>Pi serial</t>
-        </is>
-      </c>
-      <c r="U1" s="2" t="inlineStr">
-        <is>
-          <t>Power source</t>
-        </is>
-      </c>
-      <c r="V1" s="2" t="inlineStr">
-        <is>
-          <t>Network</t>
-        </is>
-      </c>
-      <c r="W1" s="2" t="inlineStr">
-        <is>
-          <t>Label applied?</t>
-        </is>
-      </c>
-      <c r="X1" s="2" t="inlineStr">
-        <is>
-          <t>Condition</t>
-        </is>
-      </c>
       <c r="Y1" s="2" t="inlineStr">
         <is>
-          <t>Issues found</t>
+          <t>Issues / notes</t>
         </is>
       </c>
       <c r="Z1" s="2" t="inlineStr">
         <is>
-          <t>Photo taken?</t>
+          <t>Audited by</t>
         </is>
       </c>
       <c r="AA1" s="2" t="inlineStr">
         <is>
-          <t>Audited by</t>
-        </is>
-      </c>
-      <c r="AB1" s="2" t="inlineStr">
-        <is>
           <t>Date</t>
-        </is>
-      </c>
-      <c r="AC1" s="2" t="inlineStr">
-        <is>
-          <t>Notes</t>
         </is>
       </c>
     </row>
@@ -723,8 +711,6 @@
       <c r="Y2" s="4" t="inlineStr"/>
       <c r="Z2" s="4" t="inlineStr"/>
       <c r="AA2" s="4" t="inlineStr"/>
-      <c r="AB2" s="4" t="inlineStr"/>
-      <c r="AC2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
@@ -786,8 +772,6 @@
       <c r="Y3" s="4" t="inlineStr"/>
       <c r="Z3" s="4" t="inlineStr"/>
       <c r="AA3" s="4" t="inlineStr"/>
-      <c r="AB3" s="4" t="inlineStr"/>
-      <c r="AC3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
@@ -853,8 +837,6 @@
       <c r="Y4" s="4" t="inlineStr"/>
       <c r="Z4" s="4" t="inlineStr"/>
       <c r="AA4" s="4" t="inlineStr"/>
-      <c r="AB4" s="4" t="inlineStr"/>
-      <c r="AC4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
@@ -920,8 +902,6 @@
       <c r="Y5" s="4" t="inlineStr"/>
       <c r="Z5" s="4" t="inlineStr"/>
       <c r="AA5" s="4" t="inlineStr"/>
-      <c r="AB5" s="4" t="inlineStr"/>
-      <c r="AC5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
@@ -983,8 +963,6 @@
       <c r="Y6" s="4" t="inlineStr"/>
       <c r="Z6" s="4" t="inlineStr"/>
       <c r="AA6" s="4" t="inlineStr"/>
-      <c r="AB6" s="4" t="inlineStr"/>
-      <c r="AC6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
@@ -1050,8 +1028,6 @@
       <c r="Y7" s="4" t="inlineStr"/>
       <c r="Z7" s="4" t="inlineStr"/>
       <c r="AA7" s="4" t="inlineStr"/>
-      <c r="AB7" s="4" t="inlineStr"/>
-      <c r="AC7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
@@ -1117,8 +1093,6 @@
       <c r="Y8" s="4" t="inlineStr"/>
       <c r="Z8" s="4" t="inlineStr"/>
       <c r="AA8" s="4" t="inlineStr"/>
-      <c r="AB8" s="4" t="inlineStr"/>
-      <c r="AC8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
@@ -1176,8 +1150,6 @@
       <c r="Y9" s="4" t="inlineStr"/>
       <c r="Z9" s="4" t="inlineStr"/>
       <c r="AA9" s="4" t="inlineStr"/>
-      <c r="AB9" s="4" t="inlineStr"/>
-      <c r="AC9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
@@ -1243,8 +1215,6 @@
       <c r="Y10" s="4" t="inlineStr"/>
       <c r="Z10" s="4" t="inlineStr"/>
       <c r="AA10" s="4" t="inlineStr"/>
-      <c r="AB10" s="4" t="inlineStr"/>
-      <c r="AC10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
@@ -1310,8 +1280,6 @@
       <c r="Y11" s="4" t="inlineStr"/>
       <c r="Z11" s="4" t="inlineStr"/>
       <c r="AA11" s="4" t="inlineStr"/>
-      <c r="AB11" s="4" t="inlineStr"/>
-      <c r="AC11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
@@ -1369,8 +1337,6 @@
       <c r="Y12" s="4" t="inlineStr"/>
       <c r="Z12" s="4" t="inlineStr"/>
       <c r="AA12" s="4" t="inlineStr"/>
-      <c r="AB12" s="4" t="inlineStr"/>
-      <c r="AC12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
@@ -1428,8 +1394,6 @@
       <c r="Y13" s="4" t="inlineStr"/>
       <c r="Z13" s="4" t="inlineStr"/>
       <c r="AA13" s="4" t="inlineStr"/>
-      <c r="AB13" s="4" t="inlineStr"/>
-      <c r="AC13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
@@ -1487,8 +1451,6 @@
       <c r="Y14" s="4" t="inlineStr"/>
       <c r="Z14" s="4" t="inlineStr"/>
       <c r="AA14" s="4" t="inlineStr"/>
-      <c r="AB14" s="4" t="inlineStr"/>
-      <c r="AC14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
@@ -1554,8 +1516,6 @@
       <c r="Y15" s="4" t="inlineStr"/>
       <c r="Z15" s="4" t="inlineStr"/>
       <c r="AA15" s="4" t="inlineStr"/>
-      <c r="AB15" s="4" t="inlineStr"/>
-      <c r="AC15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
@@ -1617,8 +1577,6 @@
       <c r="Y16" s="4" t="inlineStr"/>
       <c r="Z16" s="4" t="inlineStr"/>
       <c r="AA16" s="4" t="inlineStr"/>
-      <c r="AB16" s="4" t="inlineStr"/>
-      <c r="AC16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
@@ -1684,8 +1642,6 @@
       <c r="Y17" s="4" t="inlineStr"/>
       <c r="Z17" s="4" t="inlineStr"/>
       <c r="AA17" s="4" t="inlineStr"/>
-      <c r="AB17" s="4" t="inlineStr"/>
-      <c r="AC17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
@@ -1751,8 +1707,6 @@
       <c r="Y18" s="4" t="inlineStr"/>
       <c r="Z18" s="4" t="inlineStr"/>
       <c r="AA18" s="4" t="inlineStr"/>
-      <c r="AB18" s="4" t="inlineStr"/>
-      <c r="AC18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
@@ -1818,8 +1772,6 @@
       <c r="Y19" s="4" t="inlineStr"/>
       <c r="Z19" s="4" t="inlineStr"/>
       <c r="AA19" s="4" t="inlineStr"/>
-      <c r="AB19" s="4" t="inlineStr"/>
-      <c r="AC19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
@@ -1881,8 +1833,6 @@
       <c r="Y20" s="4" t="inlineStr"/>
       <c r="Z20" s="4" t="inlineStr"/>
       <c r="AA20" s="4" t="inlineStr"/>
-      <c r="AB20" s="4" t="inlineStr"/>
-      <c r="AC20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
@@ -1944,8 +1894,6 @@
       <c r="Y21" s="4" t="inlineStr"/>
       <c r="Z21" s="4" t="inlineStr"/>
       <c r="AA21" s="4" t="inlineStr"/>
-      <c r="AB21" s="4" t="inlineStr"/>
-      <c r="AC21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
@@ -2011,8 +1959,6 @@
       <c r="Y22" s="4" t="inlineStr"/>
       <c r="Z22" s="4" t="inlineStr"/>
       <c r="AA22" s="4" t="inlineStr"/>
-      <c r="AB22" s="4" t="inlineStr"/>
-      <c r="AC22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
@@ -2078,8 +2024,6 @@
       <c r="Y23" s="4" t="inlineStr"/>
       <c r="Z23" s="4" t="inlineStr"/>
       <c r="AA23" s="4" t="inlineStr"/>
-      <c r="AB23" s="4" t="inlineStr"/>
-      <c r="AC23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
@@ -2141,8 +2085,6 @@
       <c r="Y24" s="4" t="inlineStr"/>
       <c r="Z24" s="4" t="inlineStr"/>
       <c r="AA24" s="4" t="inlineStr"/>
-      <c r="AB24" s="4" t="inlineStr"/>
-      <c r="AC24" s="4" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
@@ -2208,8 +2150,6 @@
       <c r="Y25" s="4" t="inlineStr"/>
       <c r="Z25" s="4" t="inlineStr"/>
       <c r="AA25" s="4" t="inlineStr"/>
-      <c r="AB25" s="4" t="inlineStr"/>
-      <c r="AC25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n">
@@ -2271,8 +2211,6 @@
       <c r="Y26" s="4" t="inlineStr"/>
       <c r="Z26" s="4" t="inlineStr"/>
       <c r="AA26" s="4" t="inlineStr"/>
-      <c r="AB26" s="4" t="inlineStr"/>
-      <c r="AC26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n">
@@ -2326,8 +2264,6 @@
       <c r="Y27" s="4" t="inlineStr"/>
       <c r="Z27" s="4" t="inlineStr"/>
       <c r="AA27" s="4" t="inlineStr"/>
-      <c r="AB27" s="4" t="inlineStr"/>
-      <c r="AC27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n">
@@ -2381,8 +2317,6 @@
       <c r="Y28" s="4" t="inlineStr"/>
       <c r="Z28" s="4" t="inlineStr"/>
       <c r="AA28" s="4" t="inlineStr"/>
-      <c r="AB28" s="4" t="inlineStr"/>
-      <c r="AC28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
@@ -2430,8 +2364,6 @@
       <c r="Y29" s="4" t="inlineStr"/>
       <c r="Z29" s="4" t="inlineStr"/>
       <c r="AA29" s="4" t="inlineStr"/>
-      <c r="AB29" s="4" t="inlineStr"/>
-      <c r="AC29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n">
@@ -2479,8 +2411,6 @@
       <c r="Y30" s="4" t="inlineStr"/>
       <c r="Z30" s="4" t="inlineStr"/>
       <c r="AA30" s="4" t="inlineStr"/>
-      <c r="AB30" s="4" t="inlineStr"/>
-      <c r="AC30" s="4" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n">
@@ -2528,8 +2458,6 @@
       <c r="Y31" s="4" t="inlineStr"/>
       <c r="Z31" s="4" t="inlineStr"/>
       <c r="AA31" s="4" t="inlineStr"/>
-      <c r="AB31" s="4" t="inlineStr"/>
-      <c r="AC31" s="4" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n">
@@ -2577,8 +2505,6 @@
       <c r="Y32" s="4" t="inlineStr"/>
       <c r="Z32" s="4" t="inlineStr"/>
       <c r="AA32" s="4" t="inlineStr"/>
-      <c r="AB32" s="4" t="inlineStr"/>
-      <c r="AC32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n">
@@ -2626,8 +2552,6 @@
       <c r="Y33" s="4" t="inlineStr"/>
       <c r="Z33" s="4" t="inlineStr"/>
       <c r="AA33" s="4" t="inlineStr"/>
-      <c r="AB33" s="4" t="inlineStr"/>
-      <c r="AC33" s="4" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n">
@@ -2675,41 +2599,33 @@
       <c r="Y34" s="4" t="inlineStr"/>
       <c r="Z34" s="4" t="inlineStr"/>
       <c r="AA34" s="4" t="inlineStr"/>
-      <c r="AB34" s="4" t="inlineStr"/>
-      <c r="AC34" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AC34"/>
-  <dataValidations count="10">
-    <dataValidation sqref="L2:L34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Screen on?" prompt="Is the display powered and showing something? 'No screen found' if the venue has no MCTV screen at all." type="list">
+  <autoFilter ref="A1:AA34"/>
+  <dataValidations count="8">
+    <dataValidation sqref="M2:M34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Card left?" prompt="Confirm you left an Exceed card so the venue knows who to call about the screen." type="list">
+      <formula1>"Yes,No - nobody available,No - card not accepted"</formula1>
+    </dataValidation>
+    <dataValidation sqref="N2:N34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Screen on?" prompt="Is the display powered and showing something? 'No screen found' if the venue has no MCTV screen at all." type="list">
       <formula1>"Yes,No,No screen found"</formula1>
     </dataValidation>
-    <dataValidation sqref="M2:M34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Content playing?" prompt="Is the MCTV loop actually advancing? Watch for at least two spot changes before answering." type="list">
+    <dataValidation sqref="O2:O34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Content playing?" prompt="Is the MCTV loop actually advancing? Watch for at least two spot changes before answering." type="list">
       <formula1>"Yes,Frozen,Black,Error / no signal"</formula1>
     </dataValidation>
-    <dataValidation sqref="Q2:Q34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Orientation" prompt="How the display is hung. Our creative is built landscape; portrait screens letterbox." type="list">
-      <formula1>"Landscape,Portrait"</formula1>
+    <dataValidation sqref="P2:P34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Power test OK?" prompt="Power the unit down and back up, and confirm it returns to playing content on its own. This is the single most useful test in the audit." type="list">
+      <formula1>"Yes,No - did not come back,Not attempted"</formula1>
     </dataValidation>
-    <dataValidation sqref="R2:R34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Mount type" prompt="How it is fixed in place. Tells us what it costs to service or replace." type="list">
-      <formula1>"Wall,Ceiling,Stand,Shelf / counter,Other"</formula1>
+    <dataValidation sqref="Q2:Q34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Connection" prompt="How the Pi reaches the internet. 'Not connected' is a finding, not a failure — record it and move on." type="list">
+      <formula1>"Wi-Fi,Ethernet,Not connected"</formula1>
     </dataValidation>
-    <dataValidation sqref="S2:S34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Pi model" prompt="Raspberry Pi generation, printed on the board. 'Other / unmarked' is a fine answer." type="list">
-      <formula1>"Pi 3,Pi 4,Pi 5,Other / unmarked"</formula1>
+    <dataValidation sqref="R2:R34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Presentation OK?" prompt="Does the installation look sharp? Screen clean and clear of debris, cables concealed, nothing hanging loose." type="list">
+      <formula1>"Yes,Wires visible,Debris / dust,Wires + debris"</formula1>
     </dataValidation>
-    <dataValidation sqref="U2:U34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Power source" prompt="What the Pi is plugged into. TV USB ports cut power with the TV and cause 'dark screen' tickets." type="list">
-      <formula1>"Wall outlet,Power strip,TV USB port,PoE,Other"</formula1>
+    <dataValidation sqref="S2:S34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Photos taken?" prompt="Two shots: one wide enough to show the screen in its setting, one close on the Pi with its label." type="list">
+      <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="V2:V34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Network" prompt="How the Pi connects. Note the SSID in Notes if it is on venue guest Wi-Fi." type="list">
-      <formula1>"Wi-Fi,Ethernet,Unknown"</formula1>
-    </dataValidation>
-    <dataValidation sqref="W2:W34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Label applied?" prompt="Confirm the MCTV license label was affixed to this unit." type="list">
+    <dataValidation sqref="U2:U34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Label applied?" prompt="Confirm the MCTV label was affixed to this unit. That label doubles as the property and contact sticker." type="list">
       <formula1>"Yes,No - Pi not reachable,No - no label for this screen"</formula1>
-    </dataValidation>
-    <dataValidation sqref="X2:X34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Condition" prompt="Overall physical state of display and Pi together." type="list">
-      <formula1>"Good,Fair,Poor,Needs replacement"</formula1>
-    </dataValidation>
-    <dataValidation sqref="Z2:Z34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Photo taken?" prompt="One wide shot of the screen in place, one close shot of the Pi with its new label." type="list">
-      <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4557,7 +4473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4574,7 +4490,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-04</t>
+          <t>Generated 2026-08-07</t>
         </is>
       </c>
     </row>
@@ -4593,216 +4509,192 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Screen on?</t>
+          <t>Spoke with</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Is the display powered and showing something? 'No screen found' if the venue has no MCTV screen at all.</t>
+          <t>Name of the manager or staff member you introduced yourself to. This becomes our contact of record for the venue.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Content playing?</t>
+          <t>Card left?</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Is the MCTV loop actually advancing? Watch for at least two spot changes before answering.</t>
+          <t>Confirm you left an Exceed card so the venue knows who to call about the screen.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>Display brand</t>
+          <t>Screen on?</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Manufacturer on the bezel or the back label (Samsung, LG, TCL, Vizio...).</t>
+          <t>Is the display powered and showing something? 'No screen found' if the venue has no MCTV screen at all.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Display model</t>
+          <t>Content playing?</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Model number from the back label. Photograph it if it is hard to read.</t>
+          <t>Is the MCTV loop actually advancing? Watch for at least two spot changes before answering.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Size (in)</t>
+          <t>Power test OK?</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Diagonal screen size in inches. The model number usually starts with it.</t>
+          <t>Power the unit down and back up, and confirm it returns to playing content on its own. This is the single most useful test in the audit.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Orientation</t>
+          <t>Connection</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>How the display is hung. Our creative is built landscape; portrait screens letterbox.</t>
+          <t>How the Pi reaches the internet. 'Not connected' is a finding, not a failure — record it and move on.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Mount type</t>
+          <t>Presentation OK?</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>How it is fixed in place. Tells us what it costs to service or replace.</t>
+          <t>Does the installation look sharp? Screen clean and clear of debris, cables concealed, nothing hanging loose.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Pi model</t>
+          <t>Photos taken?</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Raspberry Pi generation, printed on the board. 'Other / unmarked' is a fine answer.</t>
+          <t>Two shots: one wide enough to show the screen in its setting, one close on the Pi with its label.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Pi serial</t>
+          <t>License # confirmed</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Serial from the Pi's own label, not the license number. Blank if the unit cannot be reached.</t>
+          <t>Write the license number from the Pi. It is pre-filled where we have it — confirm it matches, and correct it here if it does not.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Power source</t>
+          <t>Label applied?</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>What the Pi is plugged into. TV USB ports cut power with the TV and cause 'dark screen' tickets.</t>
+          <t>Confirm the MCTV label was affixed to this unit. That label doubles as the property and contact sticker.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Network</t>
+          <t>Display brand</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>How the Pi connects. Note the SSID in Notes if it is on venue guest Wi-Fi.</t>
+          <t>Manufacturer on the bezel or the back label (Samsung, LG, TCL, Vizio...).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Label applied?</t>
+          <t>Display model</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Confirm the MCTV license label was affixed to this unit.</t>
+          <t>Model number from the back label. Photograph it if it is hard to read.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Condition</t>
+          <t>Size (in)</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Overall physical state of display and Pi together.</t>
+          <t>Diagonal screen size in inches. The model number usually starts with it.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Issues found</t>
+          <t>Issues / notes</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Anything wrong: dark screen, wrong content, damaged mount, cables exposed, blocked sightline.</t>
+          <t>Anything wrong or worth knowing: dark screen, wrong content, exposed cables, blocked sightline, awkward access.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Photo taken?</t>
+          <t>Audited by</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>One wide shot of the screen in place, one close shot of the Pi with its new label.</t>
+          <t>Technician name.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Audited by</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Technician name.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
           <t>Date of the visit (YYYY-MM-DD).</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>Anything the columns above do not cover — including who you spoke to.</t>
         </is>
       </c>
     </row>

</xml_diff>